<commit_message>
Feat: implement individual password authentication using 'pass' column in My-page.xlsx with backward compatibility and editable field in mypage
</commit_message>
<xml_diff>
--- a/My-page.xlsx
+++ b/My-page.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sbs\Documents\Antigravity\Tokeidai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9562EEF-6BC2-43D2-9339-A499EA1EF04A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46613625-322C-46A0-BCFE-E864677E746D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="855" yWindow="330" windowWidth="17265" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
   <si>
     <t>ID</t>
   </si>
@@ -95,6 +95,14 @@
   </si>
   <si>
     <t>sbs@sobun.net</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>pass</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>kou</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -133,7 +141,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -156,6 +164,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -165,7 +184,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -468,10 +489,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -496,8 +517,11 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="2" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -519,8 +543,11 @@
       <c r="G2" t="s">
         <v>13</v>
       </c>
+      <c r="I2" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -542,8 +569,11 @@
       <c r="G3" t="s">
         <v>18</v>
       </c>
+      <c r="I3">
+        <v>111</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -565,8 +595,11 @@
       <c r="G4" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" t="s">
         <v>24</v>
+      </c>
+      <c r="I4">
+        <v>7777</v>
       </c>
     </row>
   </sheetData>

</xml_diff>